<commit_message>
Changes regarding the preprocessing
</commit_message>
<xml_diff>
--- a/reports/EDA/top50_words_by_label.xlsx
+++ b/reports/EDA/top50_words_by_label.xlsx
@@ -88,9 +88,6 @@
     <t>years</t>
   </si>
   <si>
-    <t>doesn</t>
-  </si>
-  <si>
     <t>said</t>
   </si>
   <si>
@@ -127,12 +124,12 @@
     <t>hope</t>
   </si>
   <si>
+    <t>thank</t>
+  </si>
+  <si>
     <t>looking</t>
   </si>
   <si>
-    <t>thank</t>
-  </si>
-  <si>
     <t>little</t>
   </si>
   <si>
@@ -176,6 +173,9 @@
   </si>
   <si>
     <t>thought</t>
+  </si>
+  <si>
+    <t>quot</t>
   </si>
   <si>
     <t>depression</t>
@@ -813,7 +813,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>803</v>
+        <v>805</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -821,7 +821,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>662</v>
+        <v>664</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -877,7 +877,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -893,7 +893,7 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>350</v>
+        <v>353</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -941,7 +941,7 @@
         <v>18</v>
       </c>
       <c r="B18">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -949,7 +949,7 @@
         <v>19</v>
       </c>
       <c r="B19">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -973,7 +973,7 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>284</v>
+        <v>272</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -981,7 +981,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>272</v>
+        <v>261</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -989,7 +989,7 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>261</v>
+        <v>253</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -997,7 +997,7 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>253</v>
+        <v>243</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -1005,7 +1005,7 @@
         <v>26</v>
       </c>
       <c r="B26">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -1013,7 +1013,7 @@
         <v>27</v>
       </c>
       <c r="B27">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -1021,7 +1021,7 @@
         <v>28</v>
       </c>
       <c r="B28">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -1029,7 +1029,7 @@
         <v>29</v>
       </c>
       <c r="B29">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -1037,7 +1037,7 @@
         <v>30</v>
       </c>
       <c r="B30">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -1045,7 +1045,7 @@
         <v>31</v>
       </c>
       <c r="B31">
-        <v>236</v>
+        <v>231</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -1053,7 +1053,7 @@
         <v>32</v>
       </c>
       <c r="B32">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -1061,7 +1061,7 @@
         <v>33</v>
       </c>
       <c r="B33">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -1069,7 +1069,7 @@
         <v>34</v>
       </c>
       <c r="B34">
-        <v>228</v>
+        <v>220</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -1085,7 +1085,7 @@
         <v>36</v>
       </c>
       <c r="B36">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -1093,7 +1093,7 @@
         <v>37</v>
       </c>
       <c r="B37">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -1101,7 +1101,7 @@
         <v>38</v>
       </c>
       <c r="B38">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -1117,7 +1117,7 @@
         <v>40</v>
       </c>
       <c r="B40">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -1125,7 +1125,7 @@
         <v>41</v>
       </c>
       <c r="B41">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -1141,7 +1141,7 @@
         <v>43</v>
       </c>
       <c r="B43">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -1157,7 +1157,7 @@
         <v>45</v>
       </c>
       <c r="B45">
-        <v>206</v>
+        <v>202</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -1173,7 +1173,7 @@
         <v>47</v>
       </c>
       <c r="B47">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -1181,7 +1181,7 @@
         <v>48</v>
       </c>
       <c r="B48">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -1197,7 +1197,7 @@
         <v>50</v>
       </c>
       <c r="B50">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -1205,7 +1205,7 @@
         <v>51</v>
       </c>
       <c r="B51">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -1292,7 +1292,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B10">
         <v>4360</v>
@@ -1316,7 +1316,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B13">
         <v>4037</v>
@@ -1356,7 +1356,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B18">
         <v>3691</v>
@@ -1364,7 +1364,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B19">
         <v>3644</v>
@@ -1404,7 +1404,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B24">
         <v>3170</v>
@@ -1452,7 +1452,7 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B30">
         <v>2758</v>
@@ -1476,7 +1476,7 @@
     </row>
     <row r="33" spans="1:2">
       <c r="A33" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B33">
         <v>2699</v>
@@ -1500,7 +1500,7 @@
     </row>
     <row r="36" spans="1:2">
       <c r="A36" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B36">
         <v>2586</v>
@@ -1508,7 +1508,7 @@
     </row>
     <row r="37" spans="1:2">
       <c r="A37" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B37">
         <v>2544</v>
@@ -1516,7 +1516,7 @@
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B38">
         <v>2528</v>
@@ -1564,7 +1564,7 @@
     </row>
     <row r="44" spans="1:2">
       <c r="A44" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B44">
         <v>2438</v>
@@ -1588,7 +1588,7 @@
     </row>
     <row r="47" spans="1:2">
       <c r="A47" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B47">
         <v>2425</v>
@@ -1596,7 +1596,7 @@
     </row>
     <row r="48" spans="1:2">
       <c r="A48" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B48">
         <v>2355</v>
@@ -1604,7 +1604,7 @@
     </row>
     <row r="49" spans="1:2">
       <c r="A49" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B49">
         <v>2294</v>
@@ -1673,7 +1673,7 @@
         <v>53</v>
       </c>
       <c r="B5">
-        <v>4524</v>
+        <v>4526</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1718,7 +1718,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B11">
         <v>2834</v>
@@ -1742,7 +1742,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B14">
         <v>2633</v>
@@ -1774,7 +1774,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B18">
         <v>2505</v>
@@ -1809,7 +1809,7 @@
         <v>56</v>
       </c>
       <c r="B22">
-        <v>2210</v>
+        <v>2212</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -1830,7 +1830,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B25">
         <v>2032</v>
@@ -1878,7 +1878,7 @@
     </row>
     <row r="31" spans="1:2">
       <c r="A31" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B31">
         <v>1742</v>
@@ -1942,7 +1942,7 @@
     </row>
     <row r="39" spans="1:2">
       <c r="A39" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B39">
         <v>1589</v>
@@ -1950,7 +1950,7 @@
     </row>
     <row r="40" spans="1:2">
       <c r="A40" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B40">
         <v>1566</v>
@@ -1998,7 +1998,7 @@
     </row>
     <row r="46" spans="1:2">
       <c r="A46" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B46">
         <v>1511</v>
@@ -2014,7 +2014,7 @@
     </row>
     <row r="48" spans="1:2">
       <c r="A48" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B48">
         <v>1490</v>
@@ -2038,7 +2038,7 @@
     </row>
     <row r="51" spans="1:2">
       <c r="A51" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B51">
         <v>1436</v>
@@ -2184,7 +2184,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B17">
         <v>782</v>
@@ -2248,7 +2248,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B25">
         <v>681</v>
@@ -2272,7 +2272,7 @@
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B28">
         <v>653</v>
@@ -2296,7 +2296,7 @@
     </row>
     <row r="31" spans="1:2">
       <c r="A31" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B31">
         <v>625</v>
@@ -2320,7 +2320,7 @@
     </row>
     <row r="34" spans="1:2">
       <c r="A34" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B34">
         <v>595</v>
@@ -2352,7 +2352,7 @@
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B38">
         <v>563</v>
@@ -2408,7 +2408,7 @@
     </row>
     <row r="45" spans="1:2">
       <c r="A45" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B45">
         <v>505</v>
@@ -2554,7 +2554,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B11">
         <v>804</v>
@@ -2642,7 +2642,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B22">
         <v>562</v>
@@ -2682,7 +2682,7 @@
     </row>
     <row r="27" spans="1:2">
       <c r="A27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B27">
         <v>532</v>
@@ -2690,7 +2690,7 @@
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B28">
         <v>529</v>
@@ -2746,7 +2746,7 @@
     </row>
     <row r="35" spans="1:2">
       <c r="A35" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B35">
         <v>479</v>
@@ -2770,7 +2770,7 @@
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B38">
         <v>460</v>
@@ -2826,7 +2826,7 @@
     </row>
     <row r="45" spans="1:2">
       <c r="A45" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B45">
         <v>405</v>
@@ -2964,7 +2964,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B10">
         <v>485</v>
@@ -3020,7 +3020,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B17">
         <v>319</v>
@@ -3036,7 +3036,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B19">
         <v>308</v>
@@ -3044,7 +3044,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B20">
         <v>302</v>
@@ -3068,7 +3068,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B23">
         <v>293</v>
@@ -3076,7 +3076,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B24">
         <v>289</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B25">
         <v>279</v>
@@ -3132,7 +3132,7 @@
     </row>
     <row r="31" spans="1:2">
       <c r="A31" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B31">
         <v>245</v>
@@ -3148,7 +3148,7 @@
     </row>
     <row r="33" spans="1:2">
       <c r="A33" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B33">
         <v>234</v>
@@ -3188,7 +3188,7 @@
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B38">
         <v>215</v>
@@ -3204,7 +3204,7 @@
     </row>
     <row r="40" spans="1:2">
       <c r="A40" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B40">
         <v>203</v>
@@ -3244,7 +3244,7 @@
     </row>
     <row r="45" spans="1:2">
       <c r="A45" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B45">
         <v>193</v>
@@ -3284,7 +3284,7 @@
     </row>
     <row r="50" spans="1:2">
       <c r="A50" t="s">
-        <v>22</v>
+        <v>129</v>
       </c>
       <c r="B50">
         <v>190</v>
@@ -3292,10 +3292,10 @@
     </row>
     <row r="51" spans="1:2">
       <c r="A51" t="s">
-        <v>129</v>
+        <v>40</v>
       </c>
       <c r="B51">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -3366,7 +3366,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B8">
         <v>342</v>
@@ -3374,7 +3374,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B9">
         <v>331</v>
@@ -3390,7 +3390,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B11">
         <v>266</v>
@@ -3406,7 +3406,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B13">
         <v>257</v>
@@ -3446,7 +3446,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B18">
         <v>206</v>
@@ -3454,7 +3454,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B19">
         <v>205</v>
@@ -3494,7 +3494,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B24">
         <v>177</v>
@@ -3534,7 +3534,7 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B29">
         <v>163</v>
@@ -3566,7 +3566,7 @@
     </row>
     <row r="33" spans="1:2">
       <c r="A33" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B33">
         <v>157</v>
@@ -3574,7 +3574,7 @@
     </row>
     <row r="34" spans="1:2">
       <c r="A34" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B34">
         <v>154</v>
@@ -3630,7 +3630,7 @@
     </row>
     <row r="41" spans="1:2">
       <c r="A41" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B41">
         <v>138</v>
@@ -3694,7 +3694,7 @@
     </row>
     <row r="49" spans="1:2">
       <c r="A49" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B49">
         <v>128</v>
@@ -3702,7 +3702,7 @@
     </row>
     <row r="50" spans="1:2">
       <c r="A50" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B50">
         <v>121</v>

</xml_diff>